<commit_message>
update output training for 128x128
</commit_message>
<xml_diff>
--- a/Inventory_trainingOutput.XLSX
+++ b/Inventory_trainingOutput.XLSX
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git\Spectrum_sensing_base_on_Deep_learning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C23645CF-8E1F-470E-A052-3F8ED97EA84A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DBDB345-B9DD-4A5D-8AB1-793EE8C0B2E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -982,7 +982,9 @@
       <c r="B20" s="1">
         <v>12</v>
       </c>
-      <c r="C20" s="1"/>
+      <c r="C20" s="11">
+        <v>0.42909999999999998</v>
+      </c>
       <c r="D20" s="1">
         <v>1E-3</v>
       </c>

</xml_diff>